<commit_message>
add multiple api payloads and downloads TEI attribute via command line arguments
</commit_message>
<xml_diff>
--- a/sql_view_response.xlsx
+++ b/sql_view_response.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,107 +446,54 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>board_member_name_p_c</t>
+          <t>bank_name_bank_account_1</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>board_member_email_vp_vc</t>
+          <t>account_number_bank_account_1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>senior_management_name</t>
+          <t>swift_code_bank_account_1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>board_member_name_vp_vc</t>
+          <t>iban_bank_account_1</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>designation_vp_vc</t>
+          <t>bank_address_bank_account_1</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>designation_p_c</t>
+          <t>bank_name_bank_account_2</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>senior_management_email</t>
+          <t>account_number_bank_account_2</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>board_member_email_p_c</t>
+          <t>swift_code_bank_account_2</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>designation_ceo_ed_director</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Afghan Medical and Guidance Association</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-04-23</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>IPPF-AFG-005</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Mohammad Yusuf Rahmani</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>f.noori@afga.org.af</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Najibullah Karimi</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Fatima Noori</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Vice-President</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>President</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>n.karimi@afga.org.af</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>m.rahmani@afga.org.af</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
+          <t>iban_bank_account_2</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>bank_address_bank_account_2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>